<commit_message>
Added comment to each test codeunit to explain it's scope and updated ATDD sheet
</commit_message>
<xml_diff>
--- a/test/atdd scenarios/Seminar Registration - ATDD Scenarios.xlsx
+++ b/test/atdd scenarios/Seminar Registration - ATDD Scenarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f2a63c87061b9b9b/Presentations/DOK/2024/Nordic/Presentation 1 - Tip ^0 Tricks for efficient and effective test automation data setup/Code Examples/Seminar Management/test/atdd scenarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="259" documentId="13_ncr:1_{BB4C36B7-EE5C-4F78-9FD6-35C3B4ED61F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D5271BF-BFB7-45A0-A436-D15EF75657A2}"/>
+  <xr:revisionPtr revIDLastSave="285" documentId="13_ncr:1_{BB4C36B7-EE5C-4F78-9FD6-35C3B4ED61F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48A0C659-17BD-4C7B-AA7C-A3CA8FCA84A8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{37BCB399-09BD-4B93-AAF4-793E3BF59A9F}"/>
+    <workbookView xWindow="-25320" yWindow="285" windowWidth="24120" windowHeight="15990" xr2:uid="{37BCB399-09BD-4B93-AAF4-793E3BF59A9F}"/>
   </bookViews>
   <sheets>
     <sheet name="ATDD Scenarios - Posting only" sheetId="2" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="122">
   <si>
     <t>Feature</t>
   </si>
@@ -2148,7 +2148,9 @@
         <v>26</v>
       </c>
       <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
+      <c r="D32" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E32" s="18" t="s">
         <v>97</v>
       </c>
@@ -2178,6 +2180,9 @@
       <c r="B33" t="s">
         <v>26</v>
       </c>
+      <c r="D33" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F33" t="s">
         <v>11</v>
       </c>
@@ -2207,6 +2212,9 @@
       <c r="B34" t="s">
         <v>26</v>
       </c>
+      <c r="D34" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F34" t="s">
         <v>11</v>
       </c>
@@ -2236,6 +2244,9 @@
       <c r="B35" t="s">
         <v>26</v>
       </c>
+      <c r="D35" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F35" t="s">
         <v>11</v>
       </c>
@@ -2265,6 +2276,9 @@
       <c r="B36" t="s">
         <v>26</v>
       </c>
+      <c r="D36" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F36" t="s">
         <v>11</v>
       </c>
@@ -2294,6 +2308,9 @@
       <c r="B37" t="s">
         <v>26</v>
       </c>
+      <c r="D37" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F37" t="s">
         <v>11</v>
       </c>
@@ -2323,6 +2340,9 @@
       <c r="B38" t="s">
         <v>26</v>
       </c>
+      <c r="D38" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F38" t="s">
         <v>12</v>
       </c>
@@ -2352,6 +2372,9 @@
       <c r="B39" t="s">
         <v>26</v>
       </c>
+      <c r="D39" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F39" t="s">
         <v>13</v>
       </c>
@@ -2382,7 +2405,9 @@
         <v>26</v>
       </c>
       <c r="C40" s="19"/>
-      <c r="D40" s="19"/>
+      <c r="D40" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E40" s="18" t="s">
         <v>99</v>
       </c>
@@ -2412,6 +2437,9 @@
       <c r="B41" t="s">
         <v>26</v>
       </c>
+      <c r="D41" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F41" t="s">
         <v>11</v>
       </c>
@@ -2441,6 +2469,9 @@
       <c r="B42" t="s">
         <v>26</v>
       </c>
+      <c r="D42" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F42" t="s">
         <v>11</v>
       </c>
@@ -2470,6 +2501,9 @@
       <c r="B43" t="s">
         <v>26</v>
       </c>
+      <c r="D43" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F43" t="s">
         <v>11</v>
       </c>
@@ -2499,6 +2533,9 @@
       <c r="B44" t="s">
         <v>26</v>
       </c>
+      <c r="D44" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F44" t="s">
         <v>11</v>
       </c>
@@ -2528,6 +2565,9 @@
       <c r="B45" t="s">
         <v>26</v>
       </c>
+      <c r="D45" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F45" t="s">
         <v>11</v>
       </c>
@@ -2557,6 +2597,9 @@
       <c r="B46" t="s">
         <v>26</v>
       </c>
+      <c r="D46" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F46" t="s">
         <v>12</v>
       </c>
@@ -2586,6 +2629,9 @@
       <c r="B47" t="s">
         <v>26</v>
       </c>
+      <c r="D47" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F47" t="s">
         <v>13</v>
       </c>
@@ -2616,7 +2662,9 @@
         <v>26</v>
       </c>
       <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
+      <c r="D48" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E48" s="18" t="s">
         <v>104</v>
       </c>
@@ -2646,6 +2694,9 @@
       <c r="B49" t="s">
         <v>26</v>
       </c>
+      <c r="D49" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F49" t="s">
         <v>11</v>
       </c>
@@ -2675,6 +2726,9 @@
       <c r="B50" t="s">
         <v>26</v>
       </c>
+      <c r="D50" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F50" t="s">
         <v>11</v>
       </c>
@@ -2704,6 +2758,9 @@
       <c r="B51" t="s">
         <v>26</v>
       </c>
+      <c r="D51" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F51" t="s">
         <v>11</v>
       </c>
@@ -2733,6 +2790,9 @@
       <c r="B52" t="s">
         <v>26</v>
       </c>
+      <c r="D52" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F52" t="s">
         <v>11</v>
       </c>
@@ -2762,6 +2822,9 @@
       <c r="B53" t="s">
         <v>26</v>
       </c>
+      <c r="D53" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F53" t="s">
         <v>11</v>
       </c>
@@ -2791,6 +2854,9 @@
       <c r="B54" t="s">
         <v>26</v>
       </c>
+      <c r="D54" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F54" t="s">
         <v>12</v>
       </c>
@@ -2820,6 +2886,9 @@
       <c r="B55" t="s">
         <v>26</v>
       </c>
+      <c r="D55" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F55" t="s">
         <v>13</v>
       </c>
@@ -2850,7 +2919,9 @@
         <v>26</v>
       </c>
       <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
+      <c r="D56" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E56" s="18" t="s">
         <v>107</v>
       </c>
@@ -2880,6 +2951,9 @@
       <c r="B57" t="s">
         <v>26</v>
       </c>
+      <c r="D57" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F57" t="s">
         <v>11</v>
       </c>
@@ -2909,6 +2983,9 @@
       <c r="B58" t="s">
         <v>26</v>
       </c>
+      <c r="D58" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F58" t="s">
         <v>11</v>
       </c>
@@ -2938,6 +3015,9 @@
       <c r="B59" t="s">
         <v>26</v>
       </c>
+      <c r="D59" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F59" t="s">
         <v>11</v>
       </c>
@@ -2967,6 +3047,9 @@
       <c r="B60" t="s">
         <v>26</v>
       </c>
+      <c r="D60" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F60" t="s">
         <v>11</v>
       </c>
@@ -2996,6 +3079,9 @@
       <c r="B61" t="s">
         <v>26</v>
       </c>
+      <c r="D61" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F61" t="s">
         <v>11</v>
       </c>
@@ -3025,6 +3111,9 @@
       <c r="B62" t="s">
         <v>26</v>
       </c>
+      <c r="D62" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F62" t="s">
         <v>12</v>
       </c>
@@ -3054,6 +3143,9 @@
       <c r="B63" t="s">
         <v>26</v>
       </c>
+      <c r="D63" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F63" t="s">
         <v>13</v>
       </c>
@@ -3084,7 +3176,9 @@
         <v>26</v>
       </c>
       <c r="C64" s="19"/>
-      <c r="D64" s="19"/>
+      <c r="D64" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E64" s="18" t="s">
         <v>110</v>
       </c>
@@ -3114,6 +3208,9 @@
       <c r="B65" t="s">
         <v>26</v>
       </c>
+      <c r="D65" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F65" t="s">
         <v>11</v>
       </c>
@@ -3143,6 +3240,9 @@
       <c r="B66" t="s">
         <v>26</v>
       </c>
+      <c r="D66" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F66" t="s">
         <v>11</v>
       </c>
@@ -3172,6 +3272,9 @@
       <c r="B67" t="s">
         <v>26</v>
       </c>
+      <c r="D67" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F67" t="s">
         <v>11</v>
       </c>
@@ -3201,6 +3304,9 @@
       <c r="B68" t="s">
         <v>26</v>
       </c>
+      <c r="D68" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F68" t="s">
         <v>11</v>
       </c>
@@ -3230,6 +3336,9 @@
       <c r="B69" t="s">
         <v>26</v>
       </c>
+      <c r="D69" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F69" t="s">
         <v>11</v>
       </c>
@@ -3259,6 +3368,9 @@
       <c r="B70" t="s">
         <v>26</v>
       </c>
+      <c r="D70" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F70" t="s">
         <v>12</v>
       </c>
@@ -3288,6 +3400,9 @@
       <c r="B71" t="s">
         <v>26</v>
       </c>
+      <c r="D71" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F71" t="s">
         <v>13</v>
       </c>
@@ -3318,7 +3433,9 @@
         <v>26</v>
       </c>
       <c r="C72" s="19"/>
-      <c r="D72" s="19"/>
+      <c r="D72" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E72" s="18" t="s">
         <v>113</v>
       </c>
@@ -3348,6 +3465,9 @@
       <c r="B73" t="s">
         <v>26</v>
       </c>
+      <c r="D73" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F73" t="s">
         <v>11</v>
       </c>
@@ -3377,6 +3497,9 @@
       <c r="B74" t="s">
         <v>26</v>
       </c>
+      <c r="D74" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F74" t="s">
         <v>11</v>
       </c>
@@ -3406,6 +3529,9 @@
       <c r="B75" t="s">
         <v>26</v>
       </c>
+      <c r="D75" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F75" t="s">
         <v>11</v>
       </c>
@@ -3435,6 +3561,9 @@
       <c r="B76" t="s">
         <v>26</v>
       </c>
+      <c r="D76" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F76" t="s">
         <v>11</v>
       </c>
@@ -3464,6 +3593,9 @@
       <c r="B77" t="s">
         <v>26</v>
       </c>
+      <c r="D77" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F77" t="s">
         <v>11</v>
       </c>
@@ -3493,6 +3625,9 @@
       <c r="B78" t="s">
         <v>26</v>
       </c>
+      <c r="D78" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F78" t="s">
         <v>12</v>
       </c>
@@ -3522,6 +3657,9 @@
       <c r="B79" t="s">
         <v>26</v>
       </c>
+      <c r="D79" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F79" t="s">
         <v>13</v>
       </c>
@@ -3552,7 +3690,9 @@
         <v>26</v>
       </c>
       <c r="C80" s="19"/>
-      <c r="D80" s="19"/>
+      <c r="D80" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E80" s="18" t="s">
         <v>116</v>
       </c>
@@ -3582,6 +3722,9 @@
       <c r="B81" t="s">
         <v>26</v>
       </c>
+      <c r="D81" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F81" t="s">
         <v>11</v>
       </c>
@@ -3611,6 +3754,9 @@
       <c r="B82" t="s">
         <v>26</v>
       </c>
+      <c r="D82" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F82" t="s">
         <v>11</v>
       </c>
@@ -3640,6 +3786,9 @@
       <c r="B83" t="s">
         <v>26</v>
       </c>
+      <c r="D83" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F83" t="s">
         <v>11</v>
       </c>
@@ -3669,6 +3818,9 @@
       <c r="B84" t="s">
         <v>26</v>
       </c>
+      <c r="D84" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F84" t="s">
         <v>11</v>
       </c>
@@ -3698,6 +3850,9 @@
       <c r="B85" t="s">
         <v>26</v>
       </c>
+      <c r="D85" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F85" t="s">
         <v>11</v>
       </c>
@@ -3727,6 +3882,9 @@
       <c r="B86" t="s">
         <v>26</v>
       </c>
+      <c r="D86" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F86" t="s">
         <v>12</v>
       </c>
@@ -3756,6 +3914,9 @@
       <c r="B87" t="s">
         <v>26</v>
       </c>
+      <c r="D87" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F87" t="s">
         <v>13</v>
       </c>
@@ -3786,7 +3947,9 @@
         <v>26</v>
       </c>
       <c r="C88" s="19"/>
-      <c r="D88" s="19"/>
+      <c r="D88" s="19" t="s">
+        <v>14</v>
+      </c>
       <c r="E88" s="18" t="s">
         <v>121</v>
       </c>
@@ -3816,6 +3979,9 @@
       <c r="B89" t="s">
         <v>26</v>
       </c>
+      <c r="D89" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F89" t="s">
         <v>11</v>
       </c>
@@ -3845,6 +4011,9 @@
       <c r="B90" t="s">
         <v>26</v>
       </c>
+      <c r="D90" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F90" t="s">
         <v>11</v>
       </c>
@@ -3874,6 +4043,9 @@
       <c r="B91" t="s">
         <v>26</v>
       </c>
+      <c r="D91" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F91" t="s">
         <v>11</v>
       </c>
@@ -3903,6 +4075,9 @@
       <c r="B92" t="s">
         <v>26</v>
       </c>
+      <c r="D92" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F92" t="s">
         <v>11</v>
       </c>
@@ -3932,6 +4107,9 @@
       <c r="B93" t="s">
         <v>26</v>
       </c>
+      <c r="D93" s="10" t="s">
+        <v>14</v>
+      </c>
       <c r="F93" t="s">
         <v>12</v>
       </c>
@@ -3960,6 +4138,9 @@
       </c>
       <c r="B94" t="s">
         <v>26</v>
+      </c>
+      <c r="D94" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="F94" t="s">
         <v>13</v>

</xml_diff>